<commit_message>
Added new source and table, made some changes
</commit_message>
<xml_diff>
--- a/src/test/java/api/resources/testdata/API_POC.xlsx
+++ b/src/test/java/api/resources/testdata/API_POC.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\001 TSC CodeBase\PPVA_Migration_Latest\src\test\java\api\resources\testdata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\01_RandD\sahil_github\java_JSON_and_db_validation\src\test\java\api\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43327CAE-C1F4-41ED-B11E-6E24D4F648B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8F3EBF0-6D44-4F03-B524-6813AC7A86FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="871" activeTab="7" xr2:uid="{10235BCC-59A8-4E1D-BA84-A2F03EB4D41C}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="871" firstSheet="2" activeTab="2" xr2:uid="{10235BCC-59A8-4E1D-BA84-A2F03EB4D41C}"/>
   </bookViews>
   <sheets>
     <sheet name="API Response" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,8 @@
     <sheet name="analysislsmeansttest" sheetId="7" r:id="rId6"/>
     <sheet name="analysislsmeanstukey" sheetId="8" r:id="rId7"/>
     <sheet name="formulations" sheetId="9" r:id="rId8"/>
-    <sheet name="Dummy" sheetId="4" r:id="rId9"/>
+    <sheet name="Formulation Hazards" sheetId="10" r:id="rId9"/>
+    <sheet name="Dummy" sheetId="4" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2685" uniqueCount="515">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2759" uniqueCount="535">
   <si>
     <t>wf12_study_author</t>
   </si>
@@ -1589,6 +1590,66 @@
   </si>
   <si>
     <t>Mastery Flower Evo</t>
+  </si>
+  <si>
+    <t>Formulation_ID</t>
+  </si>
+  <si>
+    <t>Formulation_Code</t>
+  </si>
+  <si>
+    <t>Hazard_Category</t>
+  </si>
+  <si>
+    <t>Hazard_Type</t>
+  </si>
+  <si>
+    <t>Rating</t>
+  </si>
+  <si>
+    <t>Text</t>
+  </si>
+  <si>
+    <t>Experiment_ID</t>
+  </si>
+  <si>
+    <t>content_classification</t>
+  </si>
+  <si>
+    <t>access_level</t>
+  </si>
+  <si>
+    <t>ORAL CARE QMS: STERILE DISTILLED WATER_63_MIF_1</t>
+  </si>
+  <si>
+    <t>EU SAFETY</t>
+  </si>
+  <si>
+    <t>HAZARD(H-PHRASE)</t>
+  </si>
+  <si>
+    <t>null</t>
+  </si>
+  <si>
+    <t>No Hazard</t>
+  </si>
+  <si>
+    <t>FLOW_Formulation_Hazards_25813849_2025-05-22_085529.csv</t>
+  </si>
+  <si>
+    <t>Fabric Cleaning</t>
+  </si>
+  <si>
+    <t>FLEX</t>
+  </si>
+  <si>
+    <t>5/22/2025</t>
+  </si>
+  <si>
+    <t>2025-05-26T10:59:39.127</t>
+  </si>
+  <si>
+    <t>WF12_FormulationHazards</t>
   </si>
 </sst>
 </file>
@@ -9298,9 +9359,253 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F7E3B48-7EC8-430B-B616-05A9D02F03AF}">
+  <dimension ref="A1:AB7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="38.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="17.77734375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="25.77734375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="24.33203125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="27.88671875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="19.109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="21.88671875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="31" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="8" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="19" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="35.88671875" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="32.88671875" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="14.21875" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="13.88671875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:28" s="14" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="B1" s="14" t="s">
+        <v>46</v>
+      </c>
+      <c r="C1" s="14" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" s="14" t="s">
+        <v>50</v>
+      </c>
+      <c r="E1" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="F1" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="G1" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="H1" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="I1" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="J1" s="14" t="s">
+        <v>75</v>
+      </c>
+      <c r="K1" s="14" t="s">
+        <v>76</v>
+      </c>
+      <c r="L1" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="M1" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="N1" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="O1" s="14" t="s">
+        <v>62</v>
+      </c>
+      <c r="P1" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="Q1" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="R1" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="S1" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="T1" s="14" t="s">
+        <v>83</v>
+      </c>
+      <c r="U1" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="V1" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="W1" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="X1" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="Y1" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="Z1" s="14" t="s">
+        <v>89</v>
+      </c>
+      <c r="AA1" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="AB1" s="14" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="2" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B2" t="s">
+        <v>105</v>
+      </c>
+      <c r="C2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D2" t="s">
+        <v>106</v>
+      </c>
+      <c r="E2" t="s">
+        <v>107</v>
+      </c>
+      <c r="G2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H2" t="s">
+        <v>13</v>
+      </c>
+      <c r="I2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K2" t="s">
+        <v>21</v>
+      </c>
+      <c r="L2" t="s">
+        <v>23</v>
+      </c>
+      <c r="N2" t="s">
+        <v>17</v>
+      </c>
+      <c r="O2" t="s">
+        <v>94</v>
+      </c>
+      <c r="P2" t="s">
+        <v>95</v>
+      </c>
+      <c r="Q2" t="b">
+        <v>0</v>
+      </c>
+      <c r="R2" t="s">
+        <v>96</v>
+      </c>
+      <c r="T2" t="s">
+        <v>97</v>
+      </c>
+      <c r="U2" t="s">
+        <v>98</v>
+      </c>
+      <c r="V2" t="s">
+        <v>99</v>
+      </c>
+      <c r="W2" t="s">
+        <v>100</v>
+      </c>
+      <c r="X2" t="s">
+        <v>13</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>101</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>102</v>
+      </c>
+      <c r="AA2" s="6">
+        <v>45771</v>
+      </c>
+      <c r="AB2" s="7">
+        <v>45771.320146782411</v>
+      </c>
+    </row>
+    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>25813849</v>
+      </c>
+      <c r="B7" t="s">
+        <v>524</v>
+      </c>
+      <c r="C7" t="s">
+        <v>525</v>
+      </c>
+      <c r="D7" t="s">
+        <v>526</v>
+      </c>
+      <c r="G7" t="s">
+        <v>528</v>
+      </c>
+      <c r="H7">
+        <v>124142</v>
+      </c>
+      <c r="I7" t="s">
+        <v>529</v>
+      </c>
+      <c r="J7" t="s">
+        <v>530</v>
+      </c>
+      <c r="K7" t="s">
+        <v>531</v>
+      </c>
+      <c r="L7" t="s">
+        <v>100</v>
+      </c>
+      <c r="M7" t="s">
+        <v>101</v>
+      </c>
+      <c r="N7" t="s">
+        <v>532</v>
+      </c>
+      <c r="O7" t="s">
+        <v>533</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E03AAAB-8962-4178-8798-07831BE4EC58}">
-  <dimension ref="A1:H171"/>
+  <dimension ref="A1:H178"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.21875" bestFit="1" customWidth="1"/>
@@ -13082,6 +13387,160 @@
       </c>
       <c r="G171" s="3"/>
       <c r="H171" s="3"/>
+    </row>
+    <row r="172" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A172" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B172" s="2" t="s">
+        <v>534</v>
+      </c>
+      <c r="C172" s="2" t="s">
+        <v>515</v>
+      </c>
+      <c r="D172" s="2" t="s">
+        <v>515</v>
+      </c>
+      <c r="E172" s="2">
+        <v>0</v>
+      </c>
+      <c r="F172" s="2" t="s">
+        <v>349</v>
+      </c>
+      <c r="G172" s="2"/>
+      <c r="H172" s="2"/>
+    </row>
+    <row r="173" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A173" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B173" s="3" t="s">
+        <v>534</v>
+      </c>
+      <c r="C173" s="3" t="s">
+        <v>516</v>
+      </c>
+      <c r="D173" s="3" t="s">
+        <v>516</v>
+      </c>
+      <c r="E173" s="3">
+        <v>0</v>
+      </c>
+      <c r="F173" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="G173" s="3"/>
+      <c r="H173" s="3"/>
+    </row>
+    <row r="174" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A174" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B174" s="2" t="s">
+        <v>534</v>
+      </c>
+      <c r="C174" s="2" t="s">
+        <v>517</v>
+      </c>
+      <c r="D174" s="2" t="s">
+        <v>517</v>
+      </c>
+      <c r="E174" s="2">
+        <v>0</v>
+      </c>
+      <c r="F174" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="G174" s="2"/>
+      <c r="H174" s="2"/>
+    </row>
+    <row r="175" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A175" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B175" s="3" t="s">
+        <v>534</v>
+      </c>
+      <c r="C175" s="3" t="s">
+        <v>518</v>
+      </c>
+      <c r="D175" s="3" t="s">
+        <v>518</v>
+      </c>
+      <c r="E175" s="3">
+        <v>0</v>
+      </c>
+      <c r="F175" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="G175" s="3"/>
+      <c r="H175" s="3"/>
+    </row>
+    <row r="176" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A176" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B176" s="2" t="s">
+        <v>534</v>
+      </c>
+      <c r="C176" s="2" t="s">
+        <v>519</v>
+      </c>
+      <c r="D176" s="2" t="s">
+        <v>519</v>
+      </c>
+      <c r="E176" s="2">
+        <v>0</v>
+      </c>
+      <c r="F176" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="G176" s="2"/>
+      <c r="H176" s="2"/>
+    </row>
+    <row r="177" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A177" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B177" s="3" t="s">
+        <v>534</v>
+      </c>
+      <c r="C177" s="3" t="s">
+        <v>520</v>
+      </c>
+      <c r="D177" s="3" t="s">
+        <v>520</v>
+      </c>
+      <c r="E177" s="3">
+        <v>0</v>
+      </c>
+      <c r="F177" s="18" t="s">
+        <v>49</v>
+      </c>
+      <c r="G177" s="3"/>
+      <c r="H177" s="3"/>
+    </row>
+    <row r="178" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A178" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B178" s="2" t="s">
+        <v>534</v>
+      </c>
+      <c r="C178" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D178" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E178" s="2">
+        <v>0</v>
+      </c>
+      <c r="F178" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="G178" s="2"/>
+      <c r="H178" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -17481,201 +17940,119 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F7E3B48-7EC8-430B-B616-05A9D02F03AF}">
-  <dimension ref="A1:AB2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{375756BE-81E3-451D-8F86-D7B7117A3C86}">
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.77734375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="38.88671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6.77734375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9.5546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.88671875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="17.77734375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="25.77734375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="24.33203125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="27.88671875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="19.109375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="21.88671875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="31" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="15.109375" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="8" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="19" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="35.88671875" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="32.88671875" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="14.21875" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="45.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="4.21875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="53.77734375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.77734375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.21875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="35.88671875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.21875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="22.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" s="14" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="14" t="s">
-        <v>73</v>
-      </c>
-      <c r="B1" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="C1" s="14" t="s">
-        <v>48</v>
-      </c>
-      <c r="D1" s="14" t="s">
-        <v>50</v>
-      </c>
-      <c r="E1" s="14" t="s">
-        <v>74</v>
-      </c>
-      <c r="F1" s="14" t="s">
-        <v>52</v>
-      </c>
-      <c r="G1" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="H1" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="I1" s="14" t="s">
-        <v>55</v>
-      </c>
-      <c r="J1" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="K1" s="14" t="s">
-        <v>76</v>
-      </c>
-      <c r="L1" s="14" t="s">
-        <v>77</v>
-      </c>
-      <c r="M1" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="N1" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="O1" s="14" t="s">
-        <v>62</v>
-      </c>
-      <c r="P1" s="14" t="s">
-        <v>64</v>
-      </c>
-      <c r="Q1" s="14" t="s">
-        <v>80</v>
-      </c>
-      <c r="R1" s="14" t="s">
-        <v>81</v>
-      </c>
-      <c r="S1" s="14" t="s">
-        <v>82</v>
-      </c>
-      <c r="T1" s="14" t="s">
-        <v>83</v>
-      </c>
-      <c r="U1" s="14" t="s">
-        <v>84</v>
-      </c>
-      <c r="V1" s="14" t="s">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>515</v>
+      </c>
+      <c r="B1" t="s">
+        <v>516</v>
+      </c>
+      <c r="C1" t="s">
+        <v>517</v>
+      </c>
+      <c r="D1" t="s">
+        <v>518</v>
+      </c>
+      <c r="E1" t="s">
+        <v>519</v>
+      </c>
+      <c r="F1" t="s">
+        <v>520</v>
+      </c>
+      <c r="G1" t="s">
+        <v>39</v>
+      </c>
+      <c r="H1" t="s">
+        <v>521</v>
+      </c>
+      <c r="I1" t="s">
+        <v>87</v>
+      </c>
+      <c r="J1" t="s">
         <v>85</v>
       </c>
-      <c r="W1" s="14" t="s">
-        <v>86</v>
-      </c>
-      <c r="X1" s="14" t="s">
-        <v>87</v>
-      </c>
-      <c r="Y1" s="14" t="s">
-        <v>88</v>
-      </c>
-      <c r="Z1" s="14" t="s">
+      <c r="K1" t="s">
+        <v>522</v>
+      </c>
+      <c r="L1" t="s">
+        <v>523</v>
+      </c>
+      <c r="M1" t="s">
+        <v>90</v>
+      </c>
+      <c r="N1" t="s">
         <v>89</v>
       </c>
-      <c r="AA1" s="14" t="s">
-        <v>90</v>
-      </c>
-      <c r="AB1" s="14" t="s">
+      <c r="O1" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>103</v>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>25813849</v>
       </c>
       <c r="B2" t="s">
-        <v>105</v>
+        <v>524</v>
       </c>
       <c r="C2" t="s">
-        <v>104</v>
+        <v>525</v>
       </c>
       <c r="D2" t="s">
-        <v>106</v>
+        <v>526</v>
       </c>
       <c r="E2" t="s">
-        <v>107</v>
+        <v>527</v>
+      </c>
+      <c r="F2" t="s">
+        <v>527</v>
       </c>
       <c r="G2" t="s">
-        <v>11</v>
-      </c>
-      <c r="H2" t="s">
-        <v>13</v>
+        <v>528</v>
+      </c>
+      <c r="H2">
+        <v>124142</v>
       </c>
       <c r="I2" t="s">
-        <v>15</v>
+        <v>529</v>
       </c>
       <c r="J2" t="s">
-        <v>19</v>
+        <v>530</v>
       </c>
       <c r="K2" t="s">
-        <v>21</v>
+        <v>531</v>
       </c>
       <c r="L2" t="s">
-        <v>23</v>
+        <v>100</v>
+      </c>
+      <c r="M2" t="s">
+        <v>101</v>
       </c>
       <c r="N2" t="s">
-        <v>17</v>
+        <v>532</v>
       </c>
       <c r="O2" t="s">
-        <v>94</v>
-      </c>
-      <c r="P2" t="s">
-        <v>95</v>
-      </c>
-      <c r="Q2" t="b">
-        <v>0</v>
-      </c>
-      <c r="R2" t="s">
-        <v>96</v>
-      </c>
-      <c r="T2" t="s">
-        <v>97</v>
-      </c>
-      <c r="U2" t="s">
-        <v>98</v>
-      </c>
-      <c r="V2" t="s">
-        <v>99</v>
-      </c>
-      <c r="W2" t="s">
-        <v>100</v>
-      </c>
-      <c r="X2" t="s">
-        <v>13</v>
-      </c>
-      <c r="Y2" t="s">
-        <v>101</v>
-      </c>
-      <c r="Z2" t="s">
-        <v>102</v>
-      </c>
-      <c r="AA2" s="6">
-        <v>45771</v>
-      </c>
-      <c r="AB2" s="7">
-        <v>45771.320146782411</v>
+        <v>533</v>
       </c>
     </row>
   </sheetData>

</xml_diff>